<commit_message>
Corrige planilha pública do Atalho DP #003
</commit_message>
<xml_diff>
--- a/materiais-gratuitos/atalho-dp/003-painel-visual-ferias/planilha-ficticia-ferias.xlsx
+++ b/materiais-gratuitos/atalho-dp/003-painel-visual-ferias/planilha-ficticia-ferias.xlsx
@@ -1,3 +1,23 @@
+
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\reserva\Downloads\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C388CA79-E6FC-45B2-A915-0285885CFB90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
+  <sheets>
+    <sheet name="Base Fictícia" sheetId="1" r:id="rId1"/>
+  </sheets>
+  <calcPr calcId="0"/>
+</workbook>
+</file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="53">

</xml_diff>